<commit_message>
Fix ChartMuseum API prediction finalization
</commit_message>
<xml_diff>
--- a/results/trace_ann29_3b_annotation_comparison_greedy_temp06.xlsx
+++ b/results/trace_ann29_3b_annotation_comparison_greedy_temp06.xlsx
@@ -493,22 +493,22 @@
         <v>29</v>
       </c>
       <c r="D2" t="n">
-        <v>36.30105862068966</v>
+        <v>36.30105862068965</v>
       </c>
       <c r="E2" t="n">
         <v>37.65380344827586</v>
       </c>
       <c r="F2" t="n">
-        <v>1.352731034482759</v>
+        <v>1.352744827586207</v>
       </c>
       <c r="G2" t="n">
-        <v>37.10522622123899</v>
+        <v>37.83281242813555</v>
       </c>
       <c r="H2" t="n">
-        <v>0.8041676005493378</v>
+        <v>1.53175380744589</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.548577227036869</v>
+        <v>0.1790089798596829</v>
       </c>
     </row>
     <row r="3">
@@ -526,22 +526,22 @@
         <v>27</v>
       </c>
       <c r="D3" t="n">
-        <v>35.5611037037037</v>
+        <v>35.56110370370371</v>
       </c>
       <c r="E3" t="n">
         <v>37.72743333333334</v>
       </c>
       <c r="F3" t="n">
-        <v>2.166322222222222</v>
+        <v>2.166329629629629</v>
       </c>
       <c r="G3" t="n">
-        <v>36.21282269310576</v>
+        <v>36.99430417458724</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6517189894020535</v>
+        <v>1.433200470883535</v>
       </c>
       <c r="I3" t="n">
-        <v>-1.514610640227576</v>
+        <v>-0.7331291587460945</v>
       </c>
     </row>
     <row r="4">
@@ -559,22 +559,22 @@
         <v>29</v>
       </c>
       <c r="D4" t="n">
-        <v>32.9555551724138</v>
+        <v>33.51417586206896</v>
       </c>
       <c r="E4" t="n">
-        <v>35.89908275862069</v>
+        <v>36.60253103448276</v>
       </c>
       <c r="F4" t="n">
-        <v>2.943520689655173</v>
+        <v>3.088355172413794</v>
       </c>
       <c r="G4" t="n">
-        <v>35.64736305416392</v>
+        <v>36.26805270933633</v>
       </c>
       <c r="H4" t="n">
-        <v>2.691807881750123</v>
+        <v>2.753876847267364</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.2517197044567748</v>
+        <v>-0.3344783251464298</v>
       </c>
     </row>
     <row r="5">
@@ -592,22 +592,22 @@
         <v>27</v>
       </c>
       <c r="D5" t="n">
-        <v>33.15832222222222</v>
+        <v>33.75832222222222</v>
       </c>
       <c r="E5" t="n">
-        <v>36.15974444444444</v>
+        <v>36.9153</v>
       </c>
       <c r="F5" t="n">
-        <v>3.001414814814815</v>
+        <v>3.156977777777778</v>
       </c>
       <c r="G5" t="n">
-        <v>35.17211186629182</v>
+        <v>35.83877853295849</v>
       </c>
       <c r="H5" t="n">
-        <v>2.013789644069602</v>
+        <v>2.080456310736269</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.9876325781526211</v>
+        <v>-1.07652146704151</v>
       </c>
     </row>
   </sheetData>
@@ -621,7 +621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S32"/>
+  <dimension ref="A1:S30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -760,13 +760,13 @@
         <v>2.7</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>21.1</v>
       </c>
       <c r="K2" t="n">
-        <v>-19.4</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="L2" t="n">
-        <v>-22.1</v>
+        <v>-1</v>
       </c>
       <c r="M2" t="n">
         <v>1000</v>
@@ -1324,66 +1324,66 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>extra7</t>
+          <t>candidate24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>omni3dbench</t>
+          <t>mathvista</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Omni3DBench</t>
+          <t>MathVista</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Omni3DBench</t>
+          <t>MathVista_MINI</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>501</v>
+        <v>1000</v>
       </c>
       <c r="G10" t="n">
-        <v>35.1113</v>
+        <v>62.1</v>
       </c>
       <c r="H10" t="n">
-        <v>35.2545</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1432</v>
+        <v>3.5</v>
       </c>
       <c r="J10" t="n">
-        <v>35.39796357819613</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="K10" t="n">
-        <v>0.2866635781961335</v>
+        <v>3.800000000000004</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1434635781961333</v>
+        <v>0.3000000000000114</v>
       </c>
       <c r="M10" t="n">
-        <v>501</v>
+        <v>1000</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="O10" t="n">
-        <v>7.355289421157685</v>
+        <v>142.502</v>
       </c>
       <c r="P10" t="n">
-        <v>25</v>
+        <v>4096</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -1404,61 +1404,61 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>mathvista</t>
+          <t>cvbench_3d</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MathVista</t>
+          <t>CV-Bench 3D</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MathVista_MINI</t>
+          <t>CV-Bench-3D</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="G11" t="n">
-        <v>62.1</v>
+        <v>65.83329999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>65.59999999999999</v>
+        <v>72.41670000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>3.5</v>
+        <v>6.5833</v>
       </c>
       <c r="J11" t="n">
-        <v>65.90000000000001</v>
+        <v>68.08333333333333</v>
       </c>
       <c r="K11" t="n">
-        <v>3.800000000000004</v>
+        <v>2.250033333333334</v>
       </c>
       <c r="L11" t="n">
-        <v>0.3000000000000114</v>
+        <v>-4.333366666666677</v>
       </c>
       <c r="M11" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>llm_extracted</t>
         </is>
       </c>
       <c r="O11" t="n">
-        <v>142.502</v>
+        <v>30.45416666666667</v>
       </c>
       <c r="P11" t="n">
-        <v>4096</v>
+        <v>299</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.008999999999999999</v>
+        <v>0</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -1474,52 +1474,52 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>extra7</t>
+          <t>candidate24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>visualpuzzles</t>
+          <t>wemath</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>VisualPuzzles</t>
+          <t>WeMath</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>VisualPuzzles</t>
+          <t>WeMath_COT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>vlmevalkit_reasoning</t>
+          <t>vlmevalkit_cot_qwen32b_judge</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1168</v>
+        <v>1740</v>
       </c>
       <c r="G12" t="n">
-        <v>19.2637</v>
+        <v>51.092</v>
       </c>
       <c r="H12" t="n">
-        <v>17.637</v>
+        <v>59.9425</v>
       </c>
       <c r="I12" t="n">
-        <v>-1.6267</v>
+        <v>8.8506</v>
       </c>
       <c r="J12" t="n">
-        <v>18.83561643835617</v>
+        <v>52.81609195402299</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.428083561643831</v>
+        <v>1.724091954022988</v>
       </c>
       <c r="L12" t="n">
-        <v>1.198616438356169</v>
+        <v>-7.126408045977016</v>
       </c>
       <c r="M12" t="n">
-        <v>1168</v>
+        <v>1740</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -1527,13 +1527,13 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>354.5188356164384</v>
+        <v>145.414367816092</v>
       </c>
       <c r="P12" t="n">
         <v>4096</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.01541095890410959</v>
+        <v>0.002298850574712644</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -1554,61 +1554,61 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>cvbench_3d</t>
+          <t>mathvision</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CV-Bench 3D</t>
+          <t>MathVision</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CV-Bench-3D</t>
+          <t>MathVision</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1200</v>
+        <v>3040</v>
       </c>
       <c r="G13" t="n">
-        <v>65.83329999999999</v>
+        <v>22.4671</v>
       </c>
       <c r="H13" t="n">
-        <v>72.41670000000001</v>
+        <v>26.3816</v>
       </c>
       <c r="I13" t="n">
-        <v>6.5833</v>
+        <v>3.9145</v>
       </c>
       <c r="J13" t="n">
-        <v>68.08333333333333</v>
+        <v>21.67763157894737</v>
       </c>
       <c r="K13" t="n">
-        <v>2.250033333333334</v>
+        <v>-0.7894684210526286</v>
       </c>
       <c r="L13" t="n">
-        <v>-4.333366666666677</v>
+        <v>-4.703968421052629</v>
       </c>
       <c r="M13" t="n">
-        <v>1200</v>
+        <v>3040</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>llm_extracted</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="O13" t="n">
-        <v>30.45416666666667</v>
+        <v>536.610197368421</v>
       </c>
       <c r="P13" t="n">
-        <v>299</v>
+        <v>4096</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>0.04177631578947368</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -1629,47 +1629,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>wemath</t>
+          <t>erqa</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>WeMath</t>
+          <t>ERQA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>WeMath_COT</t>
+          <t>ERQA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>vlmevalkit_cot_qwen32b_judge</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1740</v>
+        <v>400</v>
       </c>
       <c r="G14" t="n">
-        <v>51.092</v>
+        <v>38</v>
       </c>
       <c r="H14" t="n">
-        <v>59.9425</v>
+        <v>35.5</v>
       </c>
       <c r="I14" t="n">
-        <v>8.8506</v>
+        <v>-2.5</v>
       </c>
       <c r="J14" t="n">
-        <v>52.81609195402299</v>
+        <v>37.25</v>
       </c>
       <c r="K14" t="n">
-        <v>1.724091954022988</v>
+        <v>-0.75</v>
       </c>
       <c r="L14" t="n">
-        <v>-7.126408045977016</v>
+        <v>1.75</v>
       </c>
       <c r="M14" t="n">
-        <v>1740</v>
+        <v>400</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -1677,13 +1677,13 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>145.414367816092</v>
+        <v>2.035</v>
       </c>
       <c r="P14" t="n">
-        <v>4096</v>
+        <v>3</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.002298850574712644</v>
+        <v>0</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -1704,61 +1704,61 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>mathvision</t>
+          <t>treebench</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MathVision</t>
+          <t>TreeBench</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MathVision</t>
+          <t>TreeBench</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>3040</v>
+        <v>405</v>
       </c>
       <c r="G15" t="n">
-        <v>22.4671</v>
+        <v>39.7531</v>
       </c>
       <c r="H15" t="n">
-        <v>26.3816</v>
+        <v>41.2346</v>
       </c>
       <c r="I15" t="n">
-        <v>3.9145</v>
+        <v>1.4815</v>
       </c>
       <c r="J15" t="n">
-        <v>21.67763157894737</v>
+        <v>39.01234567901234</v>
       </c>
       <c r="K15" t="n">
-        <v>-0.7894684210526286</v>
+        <v>-0.7407543209876621</v>
       </c>
       <c r="L15" t="n">
-        <v>-4.703968421052629</v>
+        <v>-2.222254320987659</v>
       </c>
       <c r="M15" t="n">
-        <v>3040</v>
+        <v>405</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>llm_extracted</t>
         </is>
       </c>
       <c r="O15" t="n">
-        <v>536.610197368421</v>
+        <v>11.67407407407407</v>
       </c>
       <c r="P15" t="n">
-        <v>4096</v>
+        <v>189</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.04177631578947368</v>
+        <v>0</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -1779,17 +1779,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>erqa</t>
+          <t>countbenchqa</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ERQA</t>
+          <t>CountBenchQA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ERQA</t>
+          <t>CountBenchQA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1798,28 +1798,28 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>400</v>
+        <v>487</v>
       </c>
       <c r="G16" t="n">
-        <v>38</v>
+        <v>71.2526</v>
       </c>
       <c r="H16" t="n">
-        <v>35.5</v>
+        <v>72.4846</v>
       </c>
       <c r="I16" t="n">
-        <v>-2.5</v>
+        <v>1.232</v>
       </c>
       <c r="J16" t="n">
-        <v>37.25</v>
+        <v>77.82340862422998</v>
       </c>
       <c r="K16" t="n">
-        <v>-0.75</v>
+        <v>6.570808624229983</v>
       </c>
       <c r="L16" t="n">
-        <v>1.75</v>
+        <v>5.338808624229983</v>
       </c>
       <c r="M16" t="n">
-        <v>400</v>
+        <v>487</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>2.035</v>
+        <v>2.084188911704312</v>
       </c>
       <c r="P16" t="n">
         <v>3</v>
@@ -1854,61 +1854,61 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>treebench</t>
+          <t>mathverse</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>TreeBench</t>
+          <t>MathVerse</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TreeBench</t>
+          <t>MathVerse_MINI_Vision_Only_cot</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>405</v>
+        <v>788</v>
       </c>
       <c r="G17" t="n">
-        <v>39.7531</v>
+        <v>17.8934</v>
       </c>
       <c r="H17" t="n">
-        <v>41.2346</v>
+        <v>21.5736</v>
       </c>
       <c r="I17" t="n">
-        <v>1.4815</v>
+        <v>3.6802</v>
       </c>
       <c r="J17" t="n">
-        <v>39.01234567901234</v>
+        <v>19.54314720812183</v>
       </c>
       <c r="K17" t="n">
-        <v>-0.7407543209876621</v>
+        <v>1.649747208121831</v>
       </c>
       <c r="L17" t="n">
-        <v>-2.222254320987659</v>
+        <v>-2.030452791878169</v>
       </c>
       <c r="M17" t="n">
-        <v>405</v>
+        <v>788</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>llm_extracted</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="O17" t="n">
-        <v>11.67407407407407</v>
+        <v>496.1687817258883</v>
       </c>
       <c r="P17" t="n">
-        <v>189</v>
+        <v>4096</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>0.03426395939086294</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
@@ -1929,61 +1929,61 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>countbenchqa</t>
+          <t>charxivreason</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CountBenchQA</t>
+          <t>CharXivReason</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CountBenchQA</t>
+          <t>CharXiv_reasoning_val</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>487</v>
+        <v>1000</v>
       </c>
       <c r="G18" t="n">
-        <v>71.2526</v>
+        <v>32.7</v>
       </c>
       <c r="H18" t="n">
-        <v>72.4846</v>
+        <v>36.7</v>
       </c>
       <c r="I18" t="n">
-        <v>1.232</v>
+        <v>4</v>
       </c>
       <c r="J18" t="n">
-        <v>77.82340862422998</v>
+        <v>34.9</v>
       </c>
       <c r="K18" t="n">
-        <v>6.570808624229983</v>
+        <v>2.199999999999996</v>
       </c>
       <c r="L18" t="n">
-        <v>5.338808624229983</v>
+        <v>-1.800000000000004</v>
       </c>
       <c r="M18" t="n">
-        <v>487</v>
+        <v>1000</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>llm_extracted</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="O18" t="n">
-        <v>2.084188911704312</v>
+        <v>15.373</v>
       </c>
       <c r="P18" t="n">
-        <v>3</v>
+        <v>4096</v>
       </c>
       <c r="Q18" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
@@ -2004,61 +2004,61 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>mathverse</t>
+          <t>phyx_mini_mc</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MathVerse</t>
+          <t>PhyX mini MC</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MathVerse_MINI_Vision_Only_cot</t>
+          <t>PhyX_mini_MC</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>788</v>
+        <v>1000</v>
       </c>
       <c r="G19" t="n">
-        <v>17.8934</v>
+        <v>33.2</v>
       </c>
       <c r="H19" t="n">
-        <v>21.5736</v>
+        <v>35.6</v>
       </c>
       <c r="I19" t="n">
-        <v>3.6802</v>
+        <v>2.4</v>
       </c>
       <c r="J19" t="n">
-        <v>19.54314720812183</v>
+        <v>36.8</v>
       </c>
       <c r="K19" t="n">
-        <v>1.649747208121831</v>
+        <v>3.599999999999994</v>
       </c>
       <c r="L19" t="n">
-        <v>-2.030452791878169</v>
+        <v>1.199999999999996</v>
       </c>
       <c r="M19" t="n">
-        <v>788</v>
+        <v>1000</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>llm_extracted</t>
         </is>
       </c>
       <c r="O19" t="n">
-        <v>496.1687817258883</v>
+        <v>2</v>
       </c>
       <c r="P19" t="n">
-        <v>4096</v>
+        <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.03426395939086294</v>
+        <v>0</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
@@ -2079,61 +2079,61 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>charxivreason</t>
+          <t>physics</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CharXivReason</t>
+          <t>Physics</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CharXiv_reasoning_val</t>
+          <t>Physics</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>vlmevalkit_reasoning</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1000</v>
+        <v>1297</v>
       </c>
       <c r="G20" t="n">
-        <v>32.7</v>
+        <v>21.0486</v>
       </c>
       <c r="H20" t="n">
-        <v>36.7</v>
+        <v>20.9715</v>
       </c>
       <c r="I20" t="n">
-        <v>4</v>
+        <v>-0.0771</v>
       </c>
       <c r="J20" t="n">
-        <v>34.9</v>
+        <v>19.96915959907479</v>
       </c>
       <c r="K20" t="n">
-        <v>2.199999999999996</v>
+        <v>-1.079440400925211</v>
       </c>
       <c r="L20" t="n">
-        <v>-1.800000000000004</v>
+        <v>-1.00234040092521</v>
       </c>
       <c r="M20" t="n">
-        <v>1000</v>
+        <v>1297</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>llm_extracted</t>
         </is>
       </c>
       <c r="O20" t="n">
-        <v>15.373</v>
+        <v>971.9221279876639</v>
       </c>
       <c r="P20" t="n">
         <v>4096</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.001</v>
+        <v>0.05088666152659985</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
@@ -2149,52 +2149,52 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>extra7</t>
+          <t>candidate24</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>countqa</t>
+          <t>mmmu_pro_vision</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CountQA</t>
+          <t>MMMU-ProVis</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>CountQA</t>
+          <t>MMMU_Pro_V_COT</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>vlmevalkit_cot_boxed</t>
+          <t>vlmevalkit_cot_max2048</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1528</v>
+        <v>1730</v>
       </c>
       <c r="G21" t="n">
-        <v>15.9031</v>
+        <v>29.0173</v>
       </c>
       <c r="H21" t="n">
-        <v>15.3141</v>
+        <v>30.289</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.589</v>
+        <v>1.2717</v>
       </c>
       <c r="J21" t="n">
-        <v>16.68848167539267</v>
+        <v>28.20809248554913</v>
       </c>
       <c r="K21" t="n">
-        <v>0.785381675392669</v>
+        <v>-0.8092075144508684</v>
       </c>
       <c r="L21" t="n">
-        <v>1.374381675392669</v>
+        <v>-2.080907514450871</v>
       </c>
       <c r="M21" t="n">
-        <v>1528</v>
+        <v>1730</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -2202,13 +2202,13 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>3.195026178010471</v>
+        <v>473.8179190751445</v>
       </c>
       <c r="P21" t="n">
-        <v>24</v>
+        <v>4096</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
+        <v>0.01502890173410405</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
@@ -2229,17 +2229,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>phyx_mini_mc</t>
+          <t>blink</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PhyX mini MC</t>
+          <t>Blink</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>PhyX_mini_MC</t>
+          <t>BLINK</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2248,28 +2248,28 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1000</v>
+        <v>1901</v>
       </c>
       <c r="G22" t="n">
-        <v>33.2</v>
+        <v>48.9742</v>
       </c>
       <c r="H22" t="n">
-        <v>35.6</v>
+        <v>49.7633</v>
       </c>
       <c r="I22" t="n">
-        <v>2.4</v>
+        <v>0.7891</v>
       </c>
       <c r="J22" t="n">
-        <v>36.8</v>
+        <v>49.86849026827985</v>
       </c>
       <c r="K22" t="n">
-        <v>3.599999999999994</v>
+        <v>0.8942902682798461</v>
       </c>
       <c r="L22" t="n">
-        <v>1.199999999999996</v>
+        <v>0.1051902682798485</v>
       </c>
       <c r="M22" t="n">
-        <v>1000</v>
+        <v>1901</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -2277,10 +2277,10 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>2</v>
+        <v>6.83008942661757</v>
       </c>
       <c r="P22" t="n">
-        <v>2</v>
+        <v>349</v>
       </c>
       <c r="Q22" t="n">
         <v>0</v>
@@ -2299,52 +2299,52 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>extra7</t>
+          <t>candidate24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>spbench_si_cot</t>
+          <t>vlmbias</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SPBench SI COT</t>
+          <t>VLMBias</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SPBench-SI_CoT</t>
+          <t>VLMBias</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>vlmevalkit_cot</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1009</v>
+        <v>2782</v>
       </c>
       <c r="G23" t="n">
-        <v>17.8394</v>
+        <v>19.4824</v>
       </c>
       <c r="H23" t="n">
-        <v>17.9386</v>
+        <v>19.9497</v>
       </c>
       <c r="I23" t="n">
-        <v>0.09909999999999999</v>
+        <v>0.4673</v>
       </c>
       <c r="J23" t="n">
-        <v>19.52428146679881</v>
+        <v>20.52480230050323</v>
       </c>
       <c r="K23" t="n">
-        <v>1.68488146679881</v>
+        <v>1.04240230050323</v>
       </c>
       <c r="L23" t="n">
-        <v>1.58568146679881</v>
+        <v>0.5751023005032287</v>
       </c>
       <c r="M23" t="n">
-        <v>1009</v>
+        <v>2782</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -2352,10 +2352,10 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>105.4053518334985</v>
+        <v>4.132997843278218</v>
       </c>
       <c r="P23" t="n">
-        <v>329</v>
+        <v>5</v>
       </c>
       <c r="Q23" t="n">
         <v>0</v>
@@ -2379,61 +2379,61 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>spatialvizbench_cot</t>
+          <t>omni3dbench</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SpatialVizBench COT</t>
+          <t>Omni3DBench</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>SpatialVizBench_CoT</t>
+          <t>Omni3DBench</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>vlmevalkit_cot</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1180</v>
+        <v>501</v>
       </c>
       <c r="G24" t="n">
-        <v>21.5254</v>
+        <v>35.1113</v>
       </c>
       <c r="H24" t="n">
-        <v>27.7119</v>
+        <v>35.2545</v>
       </c>
       <c r="I24" t="n">
-        <v>6.1864</v>
+        <v>0.1432</v>
       </c>
       <c r="J24" t="n">
-        <v>27.45762711864407</v>
+        <v>35.39796357819613</v>
       </c>
       <c r="K24" t="n">
-        <v>5.932227118644068</v>
+        <v>0.2866635781961335</v>
       </c>
       <c r="L24" t="n">
-        <v>-0.2542728813559307</v>
+        <v>0.1434635781961333</v>
       </c>
       <c r="M24" t="n">
-        <v>1180</v>
+        <v>501</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>llm_extracted</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="O24" t="n">
-        <v>220.8093220338983</v>
+        <v>7.355289421157685</v>
       </c>
       <c r="P24" t="n">
-        <v>4096</v>
+        <v>25</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.001694915254237288</v>
+        <v>0</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
@@ -2454,61 +2454,61 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>mmhelix</t>
+          <t>visualpuzzles</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MM-HELIX</t>
+          <t>VisualPuzzles</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>MM-HELIX</t>
+          <t>VisualPuzzles</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>vlmevalkit_boxed_defaults</t>
+          <t>vlmevalkit_reasoning</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1290</v>
+        <v>1168</v>
       </c>
       <c r="G25" t="n">
-        <v>3.3333</v>
+        <v>19.2637</v>
       </c>
       <c r="H25" t="n">
-        <v>4.1085</v>
+        <v>17.637</v>
       </c>
       <c r="I25" t="n">
-        <v>0.7752</v>
+        <v>-1.6267</v>
       </c>
       <c r="J25" t="n">
-        <v>4.573643410852712</v>
+        <v>18.83561643835617</v>
       </c>
       <c r="K25" t="n">
-        <v>1.240343410852712</v>
+        <v>-0.428083561643831</v>
       </c>
       <c r="L25" t="n">
-        <v>0.4651434108527122</v>
+        <v>1.198616438356169</v>
       </c>
       <c r="M25" t="n">
-        <v>1290</v>
+        <v>1168</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>vlmevalkit_boxed_defaults</t>
+          <t>llm_extracted</t>
         </is>
       </c>
       <c r="O25" t="n">
-        <v>424.2790697674419</v>
+        <v>354.5188356164384</v>
       </c>
       <c r="P25" t="n">
         <v>4096</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.05736434108527132</v>
+        <v>0.01541095890410959</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
@@ -2524,52 +2524,52 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>candidate24</t>
+          <t>extra7</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>physics</t>
+          <t>countqa</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Physics</t>
+          <t>CountQA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Physics</t>
+          <t>CountQA</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>vlmevalkit_reasoning</t>
+          <t>vlmevalkit_cot_boxed</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1297</v>
+        <v>1528</v>
       </c>
       <c r="G26" t="n">
-        <v>21.0486</v>
+        <v>15.9031</v>
       </c>
       <c r="H26" t="n">
-        <v>20.9715</v>
+        <v>15.3141</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.0771</v>
+        <v>-0.589</v>
       </c>
       <c r="J26" t="n">
-        <v>19.96915959907479</v>
+        <v>16.68848167539267</v>
       </c>
       <c r="K26" t="n">
-        <v>-1.079440400925211</v>
+        <v>0.785381675392669</v>
       </c>
       <c r="L26" t="n">
-        <v>-1.00234040092521</v>
+        <v>1.374381675392669</v>
       </c>
       <c r="M26" t="n">
-        <v>1297</v>
+        <v>1528</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -2577,13 +2577,13 @@
         </is>
       </c>
       <c r="O26" t="n">
-        <v>971.9221279876639</v>
+        <v>3.195026178010471</v>
       </c>
       <c r="P26" t="n">
-        <v>4096</v>
+        <v>24</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.05088666152659985</v>
+        <v>0</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
@@ -2604,61 +2604,61 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>tablevqabench</t>
+          <t>spbench_si_cot</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>TableVQABench</t>
+          <t>SPBench SI COT</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>TableVQABench</t>
+          <t>SPBench-SI_CoT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_cot</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>1500</v>
+        <v>1009</v>
       </c>
       <c r="G27" t="n">
-        <v>71.68000000000001</v>
+        <v>17.8394</v>
       </c>
       <c r="H27" t="n">
-        <v>74.5067</v>
+        <v>17.9386</v>
       </c>
       <c r="I27" t="n">
-        <v>2.8267</v>
+        <v>0.09909999999999999</v>
       </c>
       <c r="J27" t="n">
-        <v>73.5733334</v>
+        <v>19.52428146679881</v>
       </c>
       <c r="K27" t="n">
-        <v>1.893333399999989</v>
+        <v>1.68488146679881</v>
       </c>
       <c r="L27" t="n">
-        <v>-0.9333665999999994</v>
+        <v>1.58568146679881</v>
       </c>
       <c r="M27" t="n">
-        <v>1500</v>
+        <v>1009</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>llm_extracted</t>
         </is>
       </c>
       <c r="O27" t="n">
-        <v>7.208</v>
+        <v>105.4053518334985</v>
       </c>
       <c r="P27" t="n">
-        <v>4096</v>
+        <v>329</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.0006666666666666666</v>
+        <v>0</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
@@ -2674,52 +2674,52 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>candidate24</t>
+          <t>extra7</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>mmmu_pro_vision</t>
+          <t>spatialvizbench_cot</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MMMU-ProVis</t>
+          <t>SpatialVizBench COT</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>MMMU_Pro_V_COT</t>
+          <t>SpatialVizBench_CoT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>vlmevalkit_cot_max2048</t>
+          <t>vlmevalkit_cot</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>1730</v>
+        <v>1180</v>
       </c>
       <c r="G28" t="n">
-        <v>29.0173</v>
+        <v>21.5254</v>
       </c>
       <c r="H28" t="n">
-        <v>30.289</v>
+        <v>27.7119</v>
       </c>
       <c r="I28" t="n">
-        <v>1.2717</v>
+        <v>6.1864</v>
       </c>
       <c r="J28" t="n">
-        <v>28.20809248554913</v>
+        <v>27.45762711864407</v>
       </c>
       <c r="K28" t="n">
-        <v>-0.8092075144508684</v>
+        <v>5.932227118644068</v>
       </c>
       <c r="L28" t="n">
-        <v>-2.080907514450871</v>
+        <v>-0.2542728813559307</v>
       </c>
       <c r="M28" t="n">
-        <v>1730</v>
+        <v>1180</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -2727,13 +2727,13 @@
         </is>
       </c>
       <c r="O28" t="n">
-        <v>473.8179190751445</v>
+        <v>220.8093220338983</v>
       </c>
       <c r="P28" t="n">
         <v>4096</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.01502890173410405</v>
+        <v>0.001694915254237288</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
@@ -2749,66 +2749,66 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>candidate24</t>
+          <t>extra7</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>blink</t>
+          <t>mmhelix</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Blink</t>
+          <t>MM-HELIX</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>BLINK</t>
+          <t>MM-HELIX</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_boxed_defaults</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1901</v>
+        <v>1290</v>
       </c>
       <c r="G29" t="n">
-        <v>48.9742</v>
+        <v>3.3333</v>
       </c>
       <c r="H29" t="n">
-        <v>49.7633</v>
+        <v>4.1085</v>
       </c>
       <c r="I29" t="n">
-        <v>0.7891</v>
+        <v>0.7752</v>
       </c>
       <c r="J29" t="n">
-        <v>49.86849026827985</v>
+        <v>4.573643410852712</v>
       </c>
       <c r="K29" t="n">
-        <v>0.8942902682798461</v>
+        <v>1.240343410852712</v>
       </c>
       <c r="L29" t="n">
-        <v>0.1051902682798485</v>
+        <v>0.4651434108527122</v>
       </c>
       <c r="M29" t="n">
-        <v>1901</v>
+        <v>1290</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>llm_extracted</t>
+          <t>vlmevalkit_boxed_defaults</t>
         </is>
       </c>
       <c r="O29" t="n">
-        <v>6.83008942661757</v>
+        <v>424.2790697674419</v>
       </c>
       <c r="P29" t="n">
-        <v>349</v>
+        <v>4096</v>
       </c>
       <c r="Q29" t="n">
-        <v>0</v>
+        <v>0.05736434108527132</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
@@ -2824,22 +2824,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>candidate24</t>
+          <t>extra7</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>vlmbias</t>
+          <t>tablevqabench</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>VLMBias</t>
+          <t>TableVQABench</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>VLMBias</t>
+          <t>TableVQABench</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2848,42 +2848,42 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>2782</v>
+        <v>1500</v>
       </c>
       <c r="G30" t="n">
-        <v>19.4824</v>
+        <v>71.68000000000001</v>
       </c>
       <c r="H30" t="n">
-        <v>19.9497</v>
+        <v>74.5067</v>
       </c>
       <c r="I30" t="n">
-        <v>0.4673</v>
+        <v>2.8267</v>
       </c>
       <c r="J30" t="n">
-        <v>20.52480230050323</v>
+        <v>73.5733334</v>
       </c>
       <c r="K30" t="n">
-        <v>1.04240230050323</v>
+        <v>1.893333399999989</v>
       </c>
       <c r="L30" t="n">
-        <v>0.5751023005032287</v>
+        <v>-0.9333665999999994</v>
       </c>
       <c r="M30" t="n">
-        <v>2782</v>
+        <v>1500</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>llm_extracted</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="O30" t="n">
-        <v>4.132997843278218</v>
+        <v>7.208</v>
       </c>
       <c r="P30" t="n">
-        <v>5</v>
+        <v>4096</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>0.0006666666666666666</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
@@ -2895,108 +2895,6 @@
           <t>greedy</t>
         </is>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>average</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>average</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Average</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="n">
-        <v>38018</v>
-      </c>
-      <c r="G31" t="n">
-        <v>36.30105862068966</v>
-      </c>
-      <c r="H31" t="n">
-        <v>37.65380344827586</v>
-      </c>
-      <c r="I31" t="n">
-        <v>1.352731034482759</v>
-      </c>
-      <c r="J31" t="n">
-        <v>37.10522622123899</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0.8041676005493378</v>
-      </c>
-      <c r="L31" t="n">
-        <v>-0.548577227036869</v>
-      </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="n">
-        <v>159.1789214506964</v>
-      </c>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="n">
-        <v>0.008780374689468077</v>
-      </c>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>average_excl_screenspot</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>average_excl_screenspot</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Average excl. ScreenSpot</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="n">
-        <v>35165</v>
-      </c>
-      <c r="G32" t="n">
-        <v>35.5611037037037</v>
-      </c>
-      <c r="H32" t="n">
-        <v>37.72743333333334</v>
-      </c>
-      <c r="I32" t="n">
-        <v>2.166322222222222</v>
-      </c>
-      <c r="J32" t="n">
-        <v>36.21282269310576</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0.6517189894020535</v>
-      </c>
-      <c r="L32" t="n">
-        <v>-1.514610640227576</v>
-      </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="n">
-        <v>169.151191787623</v>
-      </c>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="n">
-        <v>0.009383920142840252</v>
-      </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3009,7 +2907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S32"/>
+  <dimension ref="A1:S30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3139,22 +3037,22 @@
         <v>1000</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>16.2</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>20.4</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>4.199999999999999</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="M2" t="n">
         <v>1000</v>
@@ -3712,66 +3610,66 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>extra7</t>
+          <t>candidate24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>omni3dbench</t>
+          <t>mathvista</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Omni3DBench</t>
+          <t>MathVista</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Omni3DBench</t>
+          <t>MathVista_MINI</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>501</v>
+        <v>1000</v>
       </c>
       <c r="G10" t="n">
-        <v>32.7785</v>
+        <v>61.9</v>
       </c>
       <c r="H10" t="n">
-        <v>33.7902</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>1.0117</v>
+        <v>4.7</v>
       </c>
       <c r="J10" t="n">
-        <v>34.72671342438785</v>
+        <v>64</v>
       </c>
       <c r="K10" t="n">
-        <v>1.948213424387852</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>0.9365134243878543</v>
+        <v>-2.599999999999994</v>
       </c>
       <c r="M10" t="n">
-        <v>501</v>
+        <v>1000</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="O10" t="n">
-        <v>7.463073852295409</v>
+        <v>82.491</v>
       </c>
       <c r="P10" t="n">
-        <v>13</v>
+        <v>4096</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -3792,61 +3690,61 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>mathvista</t>
+          <t>cvbench_3d</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MathVista</t>
+          <t>CV-Bench 3D</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MathVista_MINI</t>
+          <t>CV-Bench-3D</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="G11" t="n">
-        <v>61.9</v>
+        <v>57.1667</v>
       </c>
       <c r="H11" t="n">
-        <v>66.59999999999999</v>
+        <v>64.16670000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>4.7</v>
+        <v>7</v>
       </c>
       <c r="J11" t="n">
-        <v>64</v>
+        <v>62.58333333333334</v>
       </c>
       <c r="K11" t="n">
-        <v>2.100000000000001</v>
+        <v>5.416633333333344</v>
       </c>
       <c r="L11" t="n">
-        <v>-2.599999999999994</v>
+        <v>-1.583366666666663</v>
       </c>
       <c r="M11" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>llm_extracted</t>
         </is>
       </c>
       <c r="O11" t="n">
-        <v>82.491</v>
+        <v>22.43083333333333</v>
       </c>
       <c r="P11" t="n">
-        <v>4096</v>
+        <v>335</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -3862,52 +3760,52 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>extra7</t>
+          <t>candidate24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>visualpuzzles</t>
+          <t>wemath</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>VisualPuzzles</t>
+          <t>WeMath</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>VisualPuzzles</t>
+          <t>WeMath_COT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>vlmevalkit_reasoning</t>
+          <t>vlmevalkit_cot_qwen32b_judge</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1168</v>
+        <v>1740</v>
       </c>
       <c r="G12" t="n">
-        <v>16.0959</v>
+        <v>47.7011</v>
       </c>
       <c r="H12" t="n">
-        <v>18.5788</v>
+        <v>59.1954</v>
       </c>
       <c r="I12" t="n">
-        <v>2.4829</v>
+        <v>11.4943</v>
       </c>
       <c r="J12" t="n">
-        <v>17.38013698630137</v>
+        <v>51.66666666666667</v>
       </c>
       <c r="K12" t="n">
-        <v>1.284236986301369</v>
+        <v>3.965566666666675</v>
       </c>
       <c r="L12" t="n">
-        <v>-1.198663013698631</v>
+        <v>-7.528733333333328</v>
       </c>
       <c r="M12" t="n">
-        <v>1168</v>
+        <v>1740</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -3915,13 +3813,13 @@
         </is>
       </c>
       <c r="O12" t="n">
-        <v>315.9477739726028</v>
+        <v>128.8350574712644</v>
       </c>
       <c r="P12" t="n">
-        <v>4096</v>
+        <v>3501</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.00684931506849315</v>
+        <v>0</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -3942,61 +3840,61 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>cvbench_3d</t>
+          <t>mathvision</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CV-Bench 3D</t>
+          <t>MathVision</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>CV-Bench-3D</t>
+          <t>MathVision</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1200</v>
+        <v>3040</v>
       </c>
       <c r="G13" t="n">
-        <v>57.1667</v>
+        <v>19.8684</v>
       </c>
       <c r="H13" t="n">
-        <v>64.16670000000001</v>
+        <v>25.2632</v>
       </c>
       <c r="I13" t="n">
-        <v>7</v>
+        <v>5.3947</v>
       </c>
       <c r="J13" t="n">
-        <v>62.58333333333334</v>
+        <v>21.875</v>
       </c>
       <c r="K13" t="n">
-        <v>5.416633333333344</v>
+        <v>2.006599999999999</v>
       </c>
       <c r="L13" t="n">
-        <v>-1.583366666666663</v>
+        <v>-3.388200000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>1200</v>
+        <v>3040</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>llm_extracted</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="O13" t="n">
-        <v>22.43083333333333</v>
+        <v>354.0664473684211</v>
       </c>
       <c r="P13" t="n">
-        <v>335</v>
+        <v>4096</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>0.004276315789473684</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -4017,47 +3915,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>wemath</t>
+          <t>erqa</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>WeMath</t>
+          <t>ERQA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>WeMath_COT</t>
+          <t>ERQA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>vlmevalkit_cot_qwen32b_judge</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1740</v>
+        <v>400</v>
       </c>
       <c r="G14" t="n">
-        <v>47.7011</v>
+        <v>33.25</v>
       </c>
       <c r="H14" t="n">
-        <v>59.1954</v>
+        <v>34</v>
       </c>
       <c r="I14" t="n">
-        <v>11.4943</v>
+        <v>0.75</v>
       </c>
       <c r="J14" t="n">
-        <v>51.66666666666667</v>
+        <v>36.75</v>
       </c>
       <c r="K14" t="n">
-        <v>3.965566666666675</v>
+        <v>3.5</v>
       </c>
       <c r="L14" t="n">
-        <v>-7.528733333333328</v>
+        <v>2.75</v>
       </c>
       <c r="M14" t="n">
-        <v>1740</v>
+        <v>400</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -4065,10 +3963,10 @@
         </is>
       </c>
       <c r="O14" t="n">
-        <v>128.8350574712644</v>
+        <v>2.0325</v>
       </c>
       <c r="P14" t="n">
-        <v>3501</v>
+        <v>3</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -4092,61 +3990,61 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>mathvision</t>
+          <t>treebench</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MathVision</t>
+          <t>TreeBench</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MathVision</t>
+          <t>TreeBench</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>3040</v>
+        <v>405</v>
       </c>
       <c r="G15" t="n">
-        <v>19.8684</v>
+        <v>38.2716</v>
       </c>
       <c r="H15" t="n">
-        <v>25.2632</v>
+        <v>39.7531</v>
       </c>
       <c r="I15" t="n">
-        <v>5.3947</v>
+        <v>1.4815</v>
       </c>
       <c r="J15" t="n">
-        <v>21.875</v>
+        <v>38.2716049382716</v>
       </c>
       <c r="K15" t="n">
-        <v>2.006599999999999</v>
+        <v>4.93827160141791e-06</v>
       </c>
       <c r="L15" t="n">
-        <v>-3.388200000000001</v>
+        <v>-1.481495061728403</v>
       </c>
       <c r="M15" t="n">
-        <v>3040</v>
+        <v>405</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>llm_extracted</t>
         </is>
       </c>
       <c r="O15" t="n">
-        <v>354.0664473684211</v>
+        <v>6.649382716049383</v>
       </c>
       <c r="P15" t="n">
-        <v>4096</v>
+        <v>276</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.004276315789473684</v>
+        <v>0</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -4167,17 +4065,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>erqa</t>
+          <t>countbenchqa</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ERQA</t>
+          <t>CountBenchQA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ERQA</t>
+          <t>CountBenchQA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -4186,28 +4084,28 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>400</v>
+        <v>487</v>
       </c>
       <c r="G16" t="n">
-        <v>33.25</v>
+        <v>68.7885</v>
       </c>
       <c r="H16" t="n">
-        <v>34</v>
+        <v>70.0205</v>
       </c>
       <c r="I16" t="n">
-        <v>0.75</v>
+        <v>1.232</v>
       </c>
       <c r="J16" t="n">
-        <v>36.75</v>
+        <v>73.30595482546201</v>
       </c>
       <c r="K16" t="n">
-        <v>3.5</v>
+        <v>4.517454825462011</v>
       </c>
       <c r="L16" t="n">
-        <v>2.75</v>
+        <v>3.285454825462011</v>
       </c>
       <c r="M16" t="n">
-        <v>400</v>
+        <v>487</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -4215,7 +4113,7 @@
         </is>
       </c>
       <c r="O16" t="n">
-        <v>2.0325</v>
+        <v>2.092402464065708</v>
       </c>
       <c r="P16" t="n">
         <v>3</v>
@@ -4242,61 +4140,61 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>treebench</t>
+          <t>mathverse</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>TreeBench</t>
+          <t>MathVerse</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TreeBench</t>
+          <t>MathVerse_MINI_Vision_Only_cot</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>405</v>
+        <v>788</v>
       </c>
       <c r="G17" t="n">
-        <v>38.2716</v>
+        <v>19.0355</v>
       </c>
       <c r="H17" t="n">
-        <v>39.7531</v>
+        <v>21.3198</v>
       </c>
       <c r="I17" t="n">
-        <v>1.4815</v>
+        <v>2.2843</v>
       </c>
       <c r="J17" t="n">
-        <v>38.2716049382716</v>
+        <v>22.58883248730965</v>
       </c>
       <c r="K17" t="n">
-        <v>4.93827160141791e-06</v>
+        <v>3.55333248730965</v>
       </c>
       <c r="L17" t="n">
-        <v>-1.481495061728403</v>
+        <v>1.269032487309648</v>
       </c>
       <c r="M17" t="n">
-        <v>405</v>
+        <v>788</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>llm_extracted</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="O17" t="n">
-        <v>6.649382716049383</v>
+        <v>366.7068527918782</v>
       </c>
       <c r="P17" t="n">
-        <v>276</v>
+        <v>4096</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>0.003807106598984772</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
@@ -4317,58 +4215,58 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>countbenchqa</t>
+          <t>charxivreason</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CountBenchQA</t>
+          <t>CharXivReason</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CountBenchQA</t>
+          <t>CharXiv_reasoning_val</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>487</v>
+        <v>1000</v>
       </c>
       <c r="G18" t="n">
-        <v>68.7885</v>
+        <v>29.9</v>
       </c>
       <c r="H18" t="n">
-        <v>70.0205</v>
+        <v>33.7</v>
       </c>
       <c r="I18" t="n">
-        <v>1.232</v>
+        <v>3.8</v>
       </c>
       <c r="J18" t="n">
-        <v>73.30595482546201</v>
+        <v>32.7</v>
       </c>
       <c r="K18" t="n">
-        <v>4.517454825462011</v>
+        <v>2.800000000000004</v>
       </c>
       <c r="L18" t="n">
-        <v>3.285454825462011</v>
+        <v>-1</v>
       </c>
       <c r="M18" t="n">
-        <v>487</v>
+        <v>1000</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>llm_extracted</t>
+          <t>vlmevalkit_defaults_qwen32b_judge</t>
         </is>
       </c>
       <c r="O18" t="n">
-        <v>2.092402464065708</v>
+        <v>13.009</v>
       </c>
       <c r="P18" t="n">
-        <v>3</v>
+        <v>338</v>
       </c>
       <c r="Q18" t="n">
         <v>0</v>
@@ -4392,61 +4290,61 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>mathverse</t>
+          <t>phyx_mini_mc</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MathVerse</t>
+          <t>PhyX mini MC</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MathVerse_MINI_Vision_Only_cot</t>
+          <t>PhyX_mini_MC</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>788</v>
+        <v>1000</v>
       </c>
       <c r="G19" t="n">
-        <v>19.0355</v>
+        <v>32.9</v>
       </c>
       <c r="H19" t="n">
-        <v>21.3198</v>
+        <v>37.1</v>
       </c>
       <c r="I19" t="n">
-        <v>2.2843</v>
+        <v>4.2</v>
       </c>
       <c r="J19" t="n">
-        <v>22.58883248730965</v>
+        <v>33.8</v>
       </c>
       <c r="K19" t="n">
-        <v>3.55333248730965</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="L19" t="n">
-        <v>1.269032487309648</v>
+        <v>-3.300000000000004</v>
       </c>
       <c r="M19" t="n">
-        <v>788</v>
+        <v>1000</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>llm_extracted</t>
         </is>
       </c>
       <c r="O19" t="n">
-        <v>366.7068527918782</v>
+        <v>2</v>
       </c>
       <c r="P19" t="n">
-        <v>4096</v>
+        <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.003807106598984772</v>
+        <v>0</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
@@ -4467,61 +4365,61 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>charxivreason</t>
+          <t>physics</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CharXivReason</t>
+          <t>Physics</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CharXiv_reasoning_val</t>
+          <t>Physics</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>vlmevalkit_reasoning</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1000</v>
+        <v>1297</v>
       </c>
       <c r="G20" t="n">
-        <v>29.9</v>
+        <v>21.6654</v>
       </c>
       <c r="H20" t="n">
-        <v>33.7</v>
+        <v>20.8944</v>
       </c>
       <c r="I20" t="n">
-        <v>3.8</v>
+        <v>-0.771</v>
       </c>
       <c r="J20" t="n">
-        <v>32.7</v>
+        <v>20.20046260601388</v>
       </c>
       <c r="K20" t="n">
-        <v>2.800000000000004</v>
+        <v>-1.464937393986123</v>
       </c>
       <c r="L20" t="n">
-        <v>-1</v>
+        <v>-0.693937393986122</v>
       </c>
       <c r="M20" t="n">
-        <v>1000</v>
+        <v>1297</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults_qwen32b_judge</t>
+          <t>llm_extracted</t>
         </is>
       </c>
       <c r="O20" t="n">
-        <v>13.009</v>
+        <v>755.5389360061681</v>
       </c>
       <c r="P20" t="n">
-        <v>338</v>
+        <v>4096</v>
       </c>
       <c r="Q20" t="n">
-        <v>0</v>
+        <v>0.003084040092521203</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
@@ -4537,52 +4435,52 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>extra7</t>
+          <t>candidate24</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>countqa</t>
+          <t>mmmu_pro_vision</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CountQA</t>
+          <t>MMMU-ProVis</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>CountQA</t>
+          <t>MMMU_Pro_V_COT</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>vlmevalkit_cot_boxed</t>
+          <t>vlmevalkit_cot_max2048</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1528</v>
+        <v>1730</v>
       </c>
       <c r="G21" t="n">
-        <v>15.7068</v>
+        <v>26.9364</v>
       </c>
       <c r="H21" t="n">
-        <v>16.6885</v>
+        <v>31.7919</v>
       </c>
       <c r="I21" t="n">
-        <v>0.9817</v>
+        <v>4.8555</v>
       </c>
       <c r="J21" t="n">
-        <v>17.53926701570681</v>
+        <v>27.6878612716763</v>
       </c>
       <c r="K21" t="n">
-        <v>1.832467015706809</v>
+        <v>0.7514612716763018</v>
       </c>
       <c r="L21" t="n">
-        <v>0.8507670157068077</v>
+        <v>-4.104038728323697</v>
       </c>
       <c r="M21" t="n">
-        <v>1528</v>
+        <v>1730</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -4590,13 +4488,13 @@
         </is>
       </c>
       <c r="O21" t="n">
-        <v>3.467277486910995</v>
+        <v>416.8693641618497</v>
       </c>
       <c r="P21" t="n">
-        <v>24</v>
+        <v>4096</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
+        <v>0.001734104046242775</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
@@ -4617,17 +4515,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>phyx_mini_mc</t>
+          <t>blink</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PhyX mini MC</t>
+          <t>Blink</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>PhyX_mini_MC</t>
+          <t>BLINK</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -4636,28 +4534,28 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1000</v>
+        <v>1901</v>
       </c>
       <c r="G22" t="n">
-        <v>32.9</v>
+        <v>44.5555</v>
       </c>
       <c r="H22" t="n">
-        <v>37.1</v>
+        <v>46.5018</v>
       </c>
       <c r="I22" t="n">
-        <v>4.2</v>
+        <v>1.9463</v>
       </c>
       <c r="J22" t="n">
-        <v>33.8</v>
+        <v>47.02788006312467</v>
       </c>
       <c r="K22" t="n">
-        <v>0.8999999999999986</v>
+        <v>2.472380063124668</v>
       </c>
       <c r="L22" t="n">
-        <v>-3.300000000000004</v>
+        <v>0.5260800631246667</v>
       </c>
       <c r="M22" t="n">
-        <v>1000</v>
+        <v>1901</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -4665,10 +4563,10 @@
         </is>
       </c>
       <c r="O22" t="n">
-        <v>2</v>
+        <v>5.132561809573908</v>
       </c>
       <c r="P22" t="n">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="Q22" t="n">
         <v>0</v>
@@ -4687,52 +4585,52 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>extra7</t>
+          <t>candidate24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>spbench_si_cot</t>
+          <t>vlmbias</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SPBench SI COT</t>
+          <t>VLMBias</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SPBench-SI_CoT</t>
+          <t>VLMBias</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>vlmevalkit_cot</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1009</v>
+        <v>2782</v>
       </c>
       <c r="G23" t="n">
-        <v>16.1546</v>
+        <v>23.5083</v>
       </c>
       <c r="H23" t="n">
-        <v>18.5332</v>
+        <v>23.7958</v>
       </c>
       <c r="I23" t="n">
-        <v>2.3786</v>
+        <v>0.2876</v>
       </c>
       <c r="J23" t="n">
-        <v>18.63230921704658</v>
+        <v>23.79583033788641</v>
       </c>
       <c r="K23" t="n">
-        <v>2.477709217046581</v>
+        <v>0.2875303378864125</v>
       </c>
       <c r="L23" t="n">
-        <v>0.09910921704657838</v>
+        <v>3.033788641104707e-05</v>
       </c>
       <c r="M23" t="n">
-        <v>1009</v>
+        <v>2782</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -4740,10 +4638,10 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>113.2596630327056</v>
+        <v>4.122573687994249</v>
       </c>
       <c r="P23" t="n">
-        <v>326</v>
+        <v>5</v>
       </c>
       <c r="Q23" t="n">
         <v>0</v>
@@ -4767,58 +4665,58 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>spatialvizbench_cot</t>
+          <t>omni3dbench</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SpatialVizBench COT</t>
+          <t>Omni3DBench</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>SpatialVizBench_CoT</t>
+          <t>Omni3DBench</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>vlmevalkit_cot</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1180</v>
+        <v>501</v>
       </c>
       <c r="G24" t="n">
-        <v>25.8475</v>
+        <v>32.7785</v>
       </c>
       <c r="H24" t="n">
-        <v>26.7797</v>
+        <v>33.7902</v>
       </c>
       <c r="I24" t="n">
-        <v>0.9322</v>
+        <v>1.0117</v>
       </c>
       <c r="J24" t="n">
-        <v>28.13559322033898</v>
+        <v>34.72671342438785</v>
       </c>
       <c r="K24" t="n">
-        <v>2.288093220338979</v>
+        <v>1.948213424387852</v>
       </c>
       <c r="L24" t="n">
-        <v>1.355893220338981</v>
+        <v>0.9365134243878543</v>
       </c>
       <c r="M24" t="n">
-        <v>1180</v>
+        <v>501</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>llm_extracted</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="O24" t="n">
-        <v>214.3161016949153</v>
+        <v>7.463073852295409</v>
       </c>
       <c r="P24" t="n">
-        <v>1694</v>
+        <v>13</v>
       </c>
       <c r="Q24" t="n">
         <v>0</v>
@@ -4842,61 +4740,61 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>mmhelix</t>
+          <t>visualpuzzles</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MM-HELIX</t>
+          <t>VisualPuzzles</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>MM-HELIX</t>
+          <t>VisualPuzzles</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>vlmevalkit_boxed_defaults</t>
+          <t>vlmevalkit_reasoning</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1290</v>
+        <v>1168</v>
       </c>
       <c r="G25" t="n">
-        <v>4.031</v>
+        <v>16.0959</v>
       </c>
       <c r="H25" t="n">
-        <v>4.8837</v>
+        <v>18.5788</v>
       </c>
       <c r="I25" t="n">
-        <v>0.8527</v>
+        <v>2.4829</v>
       </c>
       <c r="J25" t="n">
-        <v>3.333333333333332</v>
+        <v>17.38013698630137</v>
       </c>
       <c r="K25" t="n">
-        <v>-0.6976666666666675</v>
+        <v>1.284236986301369</v>
       </c>
       <c r="L25" t="n">
-        <v>-1.550366666666668</v>
+        <v>-1.198663013698631</v>
       </c>
       <c r="M25" t="n">
-        <v>1290</v>
+        <v>1168</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>vlmevalkit_boxed_defaults</t>
+          <t>llm_extracted</t>
         </is>
       </c>
       <c r="O25" t="n">
-        <v>265.5348837209302</v>
+        <v>315.9477739726028</v>
       </c>
       <c r="P25" t="n">
         <v>4096</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.02403100775193798</v>
+        <v>0.00684931506849315</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
@@ -4912,52 +4810,52 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>candidate24</t>
+          <t>extra7</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>physics</t>
+          <t>countqa</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Physics</t>
+          <t>CountQA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Physics</t>
+          <t>CountQA</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>vlmevalkit_reasoning</t>
+          <t>vlmevalkit_cot_boxed</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1297</v>
+        <v>1528</v>
       </c>
       <c r="G26" t="n">
-        <v>21.6654</v>
+        <v>15.7068</v>
       </c>
       <c r="H26" t="n">
-        <v>20.8944</v>
+        <v>16.6885</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.771</v>
+        <v>0.9817</v>
       </c>
       <c r="J26" t="n">
-        <v>20.20046260601388</v>
+        <v>17.53926701570681</v>
       </c>
       <c r="K26" t="n">
-        <v>-1.464937393986123</v>
+        <v>1.832467015706809</v>
       </c>
       <c r="L26" t="n">
-        <v>-0.693937393986122</v>
+        <v>0.8507670157068077</v>
       </c>
       <c r="M26" t="n">
-        <v>1297</v>
+        <v>1528</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -4965,13 +4863,13 @@
         </is>
       </c>
       <c r="O26" t="n">
-        <v>755.5389360061681</v>
+        <v>3.467277486910995</v>
       </c>
       <c r="P26" t="n">
-        <v>4096</v>
+        <v>24</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.003084040092521203</v>
+        <v>0</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
@@ -4992,58 +4890,58 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>tablevqabench</t>
+          <t>spbench_si_cot</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>TableVQABench</t>
+          <t>SPBench SI COT</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>TableVQABench</t>
+          <t>SPBench-SI_CoT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_cot</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>1500</v>
+        <v>1009</v>
       </c>
       <c r="G27" t="n">
-        <v>68.4533</v>
+        <v>16.1546</v>
       </c>
       <c r="H27" t="n">
-        <v>71.30670000000001</v>
+        <v>18.5332</v>
       </c>
       <c r="I27" t="n">
-        <v>2.8533</v>
+        <v>2.3786</v>
       </c>
       <c r="J27" t="n">
-        <v>72.48</v>
+        <v>18.63230921704658</v>
       </c>
       <c r="K27" t="n">
-        <v>4.026700000000005</v>
+        <v>2.477709217046581</v>
       </c>
       <c r="L27" t="n">
-        <v>1.173299999999998</v>
+        <v>0.09910921704657838</v>
       </c>
       <c r="M27" t="n">
-        <v>1500</v>
+        <v>1009</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>llm_extracted</t>
         </is>
       </c>
       <c r="O27" t="n">
-        <v>4.428666666666667</v>
+        <v>113.2596630327056</v>
       </c>
       <c r="P27" t="n">
-        <v>41</v>
+        <v>326</v>
       </c>
       <c r="Q27" t="n">
         <v>0</v>
@@ -5062,52 +4960,52 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>candidate24</t>
+          <t>extra7</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>mmmu_pro_vision</t>
+          <t>spatialvizbench_cot</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MMMU-ProVis</t>
+          <t>SpatialVizBench COT</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>MMMU_Pro_V_COT</t>
+          <t>SpatialVizBench_CoT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>vlmevalkit_cot_max2048</t>
+          <t>vlmevalkit_cot</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>1730</v>
+        <v>1180</v>
       </c>
       <c r="G28" t="n">
-        <v>26.9364</v>
+        <v>25.8475</v>
       </c>
       <c r="H28" t="n">
-        <v>31.7919</v>
+        <v>26.7797</v>
       </c>
       <c r="I28" t="n">
-        <v>4.8555</v>
+        <v>0.9322</v>
       </c>
       <c r="J28" t="n">
-        <v>27.6878612716763</v>
+        <v>28.13559322033898</v>
       </c>
       <c r="K28" t="n">
-        <v>0.7514612716763018</v>
+        <v>2.288093220338979</v>
       </c>
       <c r="L28" t="n">
-        <v>-4.104038728323697</v>
+        <v>1.355893220338981</v>
       </c>
       <c r="M28" t="n">
-        <v>1730</v>
+        <v>1180</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -5115,13 +5013,13 @@
         </is>
       </c>
       <c r="O28" t="n">
-        <v>416.8693641618497</v>
+        <v>214.3161016949153</v>
       </c>
       <c r="P28" t="n">
-        <v>4096</v>
+        <v>1694</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.001734104046242775</v>
+        <v>0</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
@@ -5137,66 +5035,66 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>candidate24</t>
+          <t>extra7</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>blink</t>
+          <t>mmhelix</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Blink</t>
+          <t>MM-HELIX</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>BLINK</t>
+          <t>MM-HELIX</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>vlmevalkit_defaults</t>
+          <t>vlmevalkit_boxed_defaults</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1901</v>
+        <v>1290</v>
       </c>
       <c r="G29" t="n">
-        <v>44.5555</v>
+        <v>4.031</v>
       </c>
       <c r="H29" t="n">
-        <v>46.5018</v>
+        <v>4.8837</v>
       </c>
       <c r="I29" t="n">
-        <v>1.9463</v>
+        <v>0.8527</v>
       </c>
       <c r="J29" t="n">
-        <v>47.02788006312467</v>
+        <v>3.333333333333332</v>
       </c>
       <c r="K29" t="n">
-        <v>2.472380063124668</v>
+        <v>-0.6976666666666675</v>
       </c>
       <c r="L29" t="n">
-        <v>0.5260800631246667</v>
+        <v>-1.550366666666668</v>
       </c>
       <c r="M29" t="n">
-        <v>1901</v>
+        <v>1290</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>llm_extracted</t>
+          <t>vlmevalkit_boxed_defaults</t>
         </is>
       </c>
       <c r="O29" t="n">
-        <v>5.132561809573908</v>
+        <v>265.5348837209302</v>
       </c>
       <c r="P29" t="n">
-        <v>51</v>
+        <v>4096</v>
       </c>
       <c r="Q29" t="n">
-        <v>0</v>
+        <v>0.02403100775193798</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
@@ -5212,22 +5110,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>candidate24</t>
+          <t>extra7</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>vlmbias</t>
+          <t>tablevqabench</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>VLMBias</t>
+          <t>TableVQABench</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>VLMBias</t>
+          <t>TableVQABench</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -5236,39 +5134,39 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>2782</v>
+        <v>1500</v>
       </c>
       <c r="G30" t="n">
-        <v>23.5083</v>
+        <v>68.4533</v>
       </c>
       <c r="H30" t="n">
-        <v>23.7958</v>
+        <v>71.30670000000001</v>
       </c>
       <c r="I30" t="n">
-        <v>0.2876</v>
+        <v>2.8533</v>
       </c>
       <c r="J30" t="n">
-        <v>23.79583033788641</v>
+        <v>72.48</v>
       </c>
       <c r="K30" t="n">
-        <v>0.2875303378864125</v>
+        <v>4.026700000000005</v>
       </c>
       <c r="L30" t="n">
-        <v>3.033788641104707e-05</v>
+        <v>1.173299999999998</v>
       </c>
       <c r="M30" t="n">
-        <v>2782</v>
+        <v>1500</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>llm_extracted</t>
+          <t>vlmevalkit_defaults</t>
         </is>
       </c>
       <c r="O30" t="n">
-        <v>4.122573687994249</v>
+        <v>4.428666666666667</v>
       </c>
       <c r="P30" t="n">
-        <v>5</v>
+        <v>41</v>
       </c>
       <c r="Q30" t="n">
         <v>0</v>
@@ -5283,108 +5181,6 @@
           <t>temp06</t>
         </is>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>average</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>average</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Average</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="n">
-        <v>38018</v>
-      </c>
-      <c r="G31" t="n">
-        <v>32.9555551724138</v>
-      </c>
-      <c r="H31" t="n">
-        <v>35.89908275862069</v>
-      </c>
-      <c r="I31" t="n">
-        <v>2.943520689655173</v>
-      </c>
-      <c r="J31" t="n">
-        <v>35.64736305416392</v>
-      </c>
-      <c r="K31" t="n">
-        <v>2.691807881750123</v>
-      </c>
-      <c r="L31" t="n">
-        <v>-0.2517197044567748</v>
-      </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="n">
-        <v>123.7447310258525</v>
-      </c>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="n">
-        <v>0.001836419388906977</v>
-      </c>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>average_excl_screenspot</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>average_excl_screenspot</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Average excl. ScreenSpot</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="n">
-        <v>35165</v>
-      </c>
-      <c r="G32" t="n">
-        <v>33.15832222222222</v>
-      </c>
-      <c r="H32" t="n">
-        <v>36.15974444444444</v>
-      </c>
-      <c r="I32" t="n">
-        <v>3.001414814814815</v>
-      </c>
-      <c r="J32" t="n">
-        <v>35.17211186629182</v>
-      </c>
-      <c r="K32" t="n">
-        <v>2.013789644069602</v>
-      </c>
-      <c r="L32" t="n">
-        <v>-0.9876325781526211</v>
-      </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="n">
-        <v>131.4895156797896</v>
-      </c>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="n">
-        <v>0.001972450454751939</v>
-      </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5397,7 +5193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5415,84 +5211,72 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>annotation_model</t>
+          <t>base_results</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>maveryn/trace-qwen25vl3b-rlvr-ann-additive-0p50-sectioned-step500</t>
+          <t>results/trace_full_merged_greedy_temp06_3b7b_results.xlsx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>local_model_path</t>
+          <t>annotation_model</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>/dev/shm/trace_rlvr/merged_hf/trace-qwen25vl3b-rlvr-ann-additive-0p50-sectioned-step500</t>
+          <t>maveryn/trace-qwen25vl3b-rlvr-ann-additive-0p50-sectioned-step500</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>excluded_from_31</t>
+          <t>annotation_greedy_results</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>chartqa, visiongraph_q3</t>
+          <t>results/trace_ann29_greedy4096_results.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>benchmarks</t>
+          <t>annotation_temp06_results</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>results/trace_ann29_temp06_4096_results.xlsx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>greedy_source</t>
+          <t>excluded_benchmarks</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>results/trace_ann29_greedy4096_results.xlsx</t>
+          <t>chartqa, visiongraph_q3</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>temp06_source</t>
+          <t>chartmuseum_fix</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>results/trace_ann29_temp06_4096_results.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>baseline_source</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>results/trace_full_merged_greedy_temp06_3b7b_results.xlsx</t>
+          <t>Preserve generation row order during API finalization; refinalized and rescored ChartMuseum.</t>
         </is>
       </c>
     </row>

</xml_diff>